<commit_message>
se añade la información de TODos los productos a la fecha y además se hace un scraping de las imagenes oficiales del producto 17
</commit_message>
<xml_diff>
--- a/Products.xlsx
+++ b/Products.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyecto Astro\zona-gaming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8000BB54-2C69-49D9-9868-4B08ED88E65B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B3B3673-1D0F-4B7B-B6A8-28C405626EDD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4275" yWindow="2055" windowWidth="20115" windowHeight="11340" xr2:uid="{0CBE72FF-69DA-4304-99BE-1A2A53C4AD2D}"/>
+    <workbookView xWindow="32520" yWindow="2070" windowWidth="20115" windowHeight="11340" xr2:uid="{0CBE72FF-69DA-4304-99BE-1A2A53C4AD2D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="251">
   <si>
     <t>Tarjetas Gamer</t>
   </si>
@@ -442,6 +442,342 @@
   </si>
   <si>
     <t>Link</t>
+  </si>
+  <si>
+    <t>SIX NVME M.2 SSD PCIe 4.0-512GB m.2 2280 ssd, Read UP to 7100MB/s 512GB for Gaming PS5 Memory Storage Expansion with Heatsink, Internal Solid State Hard Drive PCIe gen 4x4 Nvme for Laptop Desktop pc</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4o6FNIm</t>
+  </si>
+  <si>
+    <t>Kingston NV3 1TB M.2 2280 NVMe SSD | PCIe 4.0 Gen 4x4 | Up to 6000 MB/s | SNV3S/1000G</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4uRL2yn</t>
+  </si>
+  <si>
+    <t>Samsung 990 PRO SSD 2TB NVMe M.2 PCIe Gen4, M.2 2280 Internal Solid State Hard Drive, Seq. Read Speeds Up to 7,450 MB/s for High End Computing, Gaming, and Heavy Duty Workstations, MZ-V9P2T0B/AM</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4o6tr2Z</t>
+  </si>
+  <si>
+    <t>Fikwot FN960 512GB M.2 NVMe SSD PCIe Gen4 x4 2280 Internal Solid State Drive with Heatsink, Up to 4,800MB/s, Dynamic SLC Cache, Compatible with PS5 Internal SSD</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4fZHiWO</t>
+  </si>
+  <si>
+    <t>KOOTION 512GB PCIe 3.0 M.2 Internal Solid State Drive PCle 3.0x4 SSD NVMe M.2 2280 Internal SSD Up to 3500MB/s PCIe Gen 3 NVMe SSD Less Heat Large Storage M.2 Internal Solid State Hard Drive for PC</t>
+  </si>
+  <si>
+    <t>https://amzn.to/3RKHCyR</t>
+  </si>
+  <si>
+    <t>WD_Black SN7100 2TB NVMe SSD - Gen4 PCIe, M.2 2280, Up to 7,250 MB/s Read Speed, Up to 6,900 MB/s Write Speed, Next Gen TLC 3D NAND, for Laptops, Handheld Gaming Devices - WDS200T4X0E</t>
+  </si>
+  <si>
+    <t>https://amzn.to/3RR3SHh</t>
+  </si>
+  <si>
+    <t>fanxiang S501Q SSD 512GB PCle 3.0x4 Internal Solid State Drive, NVMe M.2 2280 Internal Solid State Drive, SLC Cache 3D NAND Up to 3000MB/s for Laptop and PC Desktops</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4e2Vg7X</t>
+  </si>
+  <si>
+    <t>1000W Fully Modular Power Supply, 80+ Gold Certified PSU | ATX 3.1 &amp; PCIe 5.1 Ready | 12V-2x6 Connector | 140mm Low-Noise Fan | 105℃ Japanese Capacitors | Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/43kKiFR</t>
+  </si>
+  <si>
+    <t>1000W Fully Modular Power Supply, 80+ Gold PSU, ATX 3.1 &amp; PCIe 5.1 Ready, Native Dual-Color 12V-2x6 Cable, RGB Low-Noise Smart Fan, 105°C-Rated Capacitors, Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/3SmBuwJ</t>
+  </si>
+  <si>
+    <t>CORSAIR RM750e ATX 3.1 PCIe 5.1 Ready Fully Modular 750W Power Supply – 12V-2x6 Cable Included, Cybenetics Gold Efficiency, 105°C-Rated Capacitors, Modern Standby Mode – Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4ucnyml</t>
+  </si>
+  <si>
+    <t>GOLDEN FIELD 850W Power Supply - 80 Plus Gold Fully Modular ATX 3.1 &amp; PCIe 5.1 - Native 600W 12V-2x6 Cable - Japanese Capacitors - ECO Mode - LLC + DC-DC + Active PFC - 850 Watt Gaming PC PSU - NX850</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4o9nkep</t>
+  </si>
+  <si>
+    <t>Vetroo 850W Power Supply Dual PCIe 5.1 ATX 3.1 Ready, 80 Plus Gold Full Modular, Quiet Operation with 120mm FDB Fan, 10-Year Warranty - White</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4vt3ey7</t>
+  </si>
+  <si>
+    <t>ASRock PRO-650G Power Supply - 650W 80 Plus Gold Certified, ATX 3.1 Ready, 120mm Fan, Full Protection Circuit, 3-Year Warranty</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4ac6DJs</t>
+  </si>
+  <si>
+    <t>ASRock PRO 850G Power Supply - 850W 80 Plus Gold Certified, ATX 3.1 &amp; PCIe 5.1 Ready, Native 12V-2x6 Connector, 120mm Low-Noise Fan, 3-Year Warranty</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4vyUQ0g</t>
+  </si>
+  <si>
+    <t>ARCTIC Liquid Freezer III Pro 360 A-RGB - AIO CPU Cooler, 3 x 120 mm Water Cooling, 38 mm Radiator, PWM Pump, VRM Fan, AMD AM5/AM4, Intel LGA1851/1700 Contact Frame - Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4vyWVt6</t>
+  </si>
+  <si>
+    <t>ARCTIC Liquid Freezer III Pro 360 A-RGB (White) - AIO CPU Cooler, 3 x 120 mm Water Cooling, 38 mm Radiator, PWM Pump, VRM Fan, AMD AM5/AM4, Intel LGA1851/1700 Contact Frame - White</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4v1YgbR</t>
+  </si>
+  <si>
+    <t>ARCTIC Liquid Freezer III Pro 360 - AIO CPU Cooler, 3 x 120 mm Water Cooling, 38 mm Radiator, PWM Pump, VRM Fan, AMD AM5/AM4, Intel LGA1851/1700 Contact Frame - Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4dMyJgI</t>
+  </si>
+  <si>
+    <t>CORSAIR Nautilus 360 RS ARGB Liquid CPU Cooler – 360mm AIO – Low-Noise – Direct Motherboard Connection – Daisy-Chain – Intel LGA 1851/1700, AMD AM5/AM4 – 3X RS120 ARGB Fans Included – Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4e5l57h</t>
+  </si>
+  <si>
+    <t>Minorsonic AIO CPU Cooler, 360mm AIO with High-Speed Ceramic Bearing Pump, 3X PWM ARGB Fans, 3-Phase Motor for Better Cooling Performance, Heat Transfer, Low Noise, Intel LGA 1851/1700, AMD AM5/AM4</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4e8ymvW</t>
+  </si>
+  <si>
+    <t>Antec Skeleton 360 ARGB Liquid CPU Cooler, 360mm Radiator, High-Performance Pump, 3 x 120mm PWM ARGB Fans, Copper Base, Intel LGA 115X/1200/1700/20XX, AMD AM4/AM5, Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/3RLqJnG</t>
+  </si>
+  <si>
+    <t>Thermalright Aqua Elite 240 V3 Water Cooling CPU Cooler, Double PWM ARGB Fans with S-FDB Bearings,Efficient PWM Controlled Pump,for AMD/AM4/AM5, Intel LGA1150/1151/1200/2011/1700/1851, (AE240 V3)</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4dMyORy</t>
+  </si>
+  <si>
+    <t>Thermalright Peerless Assassin 120 Vision MAX ARGB White CPU Air Cooler, Twin Tower Radiator 2150RPM,480x854 Resolving Power IPS Screen with 5’’,Computer Cooler for Intel lga1851/1700/115x,AM4/AM5</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4dQ6rSz</t>
+  </si>
+  <si>
+    <t>Thermalrlght Assassin Spirit 120 EVO CPU Cooler Air with 4×6mm HeatPipes, TL-S12-S PWM Fan Heatsink CPU Cooler,156mm High, for AMD:AM4 AM5/Intel 1700/1150/1151/1200,LGA17XX PC Cooler</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4o6hIl2</t>
+  </si>
+  <si>
+    <t>Vetroo V5 CPU Air Cooler with 5 Heat Pipes 120mm FDB PWM Processor Cooling for Intel LGA 1851/1700/1200/115X AMD AM5/AM4, Addressable RGB Lights Sync - White</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4dQQ203</t>
+  </si>
+  <si>
+    <t>Noctua NH-D15 G2 HBC, Dual Tower CPU Cooler, Specialised High Base Convexity Version for Intel LGA1700 (Brown)</t>
+  </si>
+  <si>
+    <t>https://amzn.to/49KpDia</t>
+  </si>
+  <si>
+    <t>Thermalright Peerless Assassin 120 SE CPU Cooler, 6 Heat Pipes AGHP Technology, Dual 120mm PWM Fans, 1550RPM Speed, for AMD:AM4 AM5/Intel LGA 1700/1150/1151/1200/1851,PC Cooler</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4g1ZQFS</t>
+  </si>
+  <si>
+    <t>KF620-DGT CPU Air Cooler, Dual ARGB PWM Fans, 6 Heat Pipes, Digital Display Top Cover - High-Performance Cooling for AMD:AM4 AM5/Intel LGA 1700/115X/1200/1366/1851 PC Cooler(Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4of8GCy</t>
+  </si>
+  <si>
+    <t>IX20 ARGB Air Cooling Fan, Twin Tower CPU Cooler with Dual 120mm Fans, 6 Copper Heat Pipes, 6.2 Inch High for AMD AM4/AM5 and Intel LGA 115X/1200/1366/1700/1851/2011, 265W TDP (White)</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4fxCUOR</t>
+  </si>
+  <si>
+    <t>FOIFKIN F600 PC Case - Pre-Installed 7 PWM ARGB Fan, ATX Mid-Tower Gaming PC Case, 270° Panoramic Glass with Type-C, FOIFKIN (Black, F600)</t>
+  </si>
+  <si>
+    <t>https://amzn.to/49CU6Pc</t>
+  </si>
+  <si>
+    <t>RUIX OV303 ATX Mid-Tower PC Case, Pre-Installed 4 x 120mm Prism ARGB PWM Fans, USB 3.0 &amp; Type-C Ports, High-Airflow Gaming Computer Case - Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/3RPC4TJ</t>
+  </si>
+  <si>
+    <t>GAMDIAS White Mid Tower Gaming Computer Case w/Display&amp; App, ATX Tempered Glass PC Case, Built-in 3x120mm ARGB PWM Fans, Up to RTX GPU/VGA 410mm &amp; 360mm AIO/Radiator &amp; 6x120mm Fans &amp; 160mm CPU Cooler</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4vpHfIo</t>
+  </si>
+  <si>
+    <t>JONSBO TK-2 Black ATX Mid-Tower Pc Case,Hyperboloid Glass Design, Separated Cabinet Structure, Al Alloy Shell Desktop Computer Case, Support BTF Motherboard/ATX Power supply/360 AIO, Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4ea3cUX</t>
+  </si>
+  <si>
+    <t>CORSAIR 4000D RS ARGB Frame Modular Mid-Tower ATX PC Case, High Airflow, 3X Pre-Installed RS Fans, InfiniRail™ Mounting System, ASUS BTF, MSI Zero, Gigabyte Stealth, Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4dVdQ1u</t>
+  </si>
+  <si>
+    <t>Gaming PC Case, ATX Cpmputer CASE with 7 PWM ARGB Fans Pre-Installed,Type-C Full-View Dual Tempered Glass, Mid Tower Computer CASE Black, (H4)</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4o8APLt</t>
+  </si>
+  <si>
+    <t>White PC Case, ATX Gaming PC Case with 7 PWM ARGB Fans Pre-Installed,Type-C Full-View Dual Tempered Glass, Gaming Computer CASE</t>
+  </si>
+  <si>
+    <t>https://amzn.to/49JizlT</t>
+  </si>
+  <si>
+    <t>RedThunder K10 Wired Gaming Keyboard and Mouse and Wrist Rest Combo, RGB Backlit, Mechanical Feel Anti-ghosting Keyboard + 7D 7200 DPI Mice+Soft Leather Wrist Rest 3 in 1 PC Gamer Accessories(Black)</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4uf6cVO</t>
+  </si>
+  <si>
+    <t>RedThunder K75 Wireless Mechanical Gaming Keyboard, 75% Hot Swappable Creamy Keyboard with Knob, RGB Backlit, Pre-lubed Linear Switches, Side Engraved PBT Keycaps, Wireless/Wired/BT5.0, Gradient Gray</t>
+  </si>
+  <si>
+    <t>https://amzn.to/43TJ4kY</t>
+  </si>
+  <si>
+    <t>AULA F75 Pro Wireless Mechanical Keyboard,75% Hot Swappable Custom Keyboard with Knob,RGB Backlit,Pre-lubed Reaper Switches,Side Printed PBT Keycaps,2.4GHz/USB-C/BT5.0 Mechanical Gaming Keyboards</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4enLhv3</t>
+  </si>
+  <si>
+    <t>Redragon Mechanical Gaming Keyboard Wired, 11 Programmable Backlit Modes, Hot-Swappable Red Switch, Anti-Ghosting, Double-Shot PBT Keycaps, Light Up Keyboard for PC Mac</t>
+  </si>
+  <si>
+    <t>https://amzn.to/43hRWAL</t>
+  </si>
+  <si>
+    <t>AULA F75 Pro Wireless Mechanical Keyboard with Knob,75% Hot Swappable Custom Gaming Keyboards,RGB Backlit,Pre-lubed Switches,Side Printed PBT Keycaps Creamy Sounding Computer Keyboard, Line White</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4dSfYZe</t>
+  </si>
+  <si>
+    <t>M75 Mechanical Keyboard,75% Gasket Hot Swappable,RGB Backlit,Side Printed PBT Keycaps,2.4Ghz/Bluetooth/USB-C Gaming Keyboards (Black and Pink)</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4e6FNUc</t>
+  </si>
+  <si>
+    <t>AULA S75 PRO Wireless Mechanical Keyboard with Screen&amp;Knob, Tri-Mode Hot Swappable Gaming Keyboard 75%, Pre-lubed Switches, RGB Backlit, Side Printed PBT Keycaps, Creamy Sounding Computer Keyboards</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4vv1rJ4</t>
+  </si>
+  <si>
+    <t>MAMBASNAKE Attack Shark X3 Wireless Gaming Mouse, 49g Ultralight, PixArt PAW3395 26000 DPI, Bluetooth/2.4Ghz /Wired Tri-Mode, 200Hrs Rechargeable Battery, Kailh GM8.0 Switch for PC/MAC/Win Black&amp;Tape</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4o6ukIR</t>
+  </si>
+  <si>
+    <t>Pulsar Gaming Gears X3 Crazylight Wireless Gaming Mouse, Ultra Lightweight 1.51 oz (43g), Hybrid Ergonomic, Optical Switch, 32000 DPI, 750 IPS, XS-1 Sensor, 8k Compatible (Uyuni White)</t>
+  </si>
+  <si>
+    <t>https://amzn.to/3RLr9KM</t>
+  </si>
+  <si>
+    <t>azer Basilisk V3 Customizable Ergonomic Gaming Mouse: Fastest Gaming Mouse Switch - Chroma RGB Lighting - 26K DPI Optical Sensor - 11 Programmable Buttons - HyperScroll Tilt Wheel - Classic Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4ulGsaC</t>
+  </si>
+  <si>
+    <t>Razer Viper V4 Pro Wireless Esports Gaming Mouse – 49g Ultra Lightweight, Fast &amp; Precise, 50K DPI Optical Sensor, 8K Polling, Gen-4 Optical Switches, Scroll Wheel, USB-C Charging, for PC &amp; Mac – Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/3QqHeFf</t>
+  </si>
+  <si>
+    <t>GravaStar Mercury M2 Wireless Gaming Mouse with 26,000 DPI, PAW3395DM Sensor -79g Lightweight Hollowed-Out Design -5 Programmable Buttons -5 Dynamic Lightsync RGB</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4ujsZjx</t>
+  </si>
+  <si>
+    <t>DAIDAI AJAZZ AJ159P Wireless Gaming Mouse with RGB Charging Dock, PAW3395 26K DPI Sensor, 56G Lightweight Ergonomic Mouse, 5 Programmable Buttons, 80 Million ASIN Switch</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4aeSsTX</t>
+  </si>
+  <si>
+    <t>Razer Basilisk V3 X HyperSpeed Customizable Wireless Gaming Mouse: Mechanical Switches Gen-2-5G Advanced 18K Optical Sensor - Chroma RGB - 9 Programmable Controls - 285 Hr Battery - Classic Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4vvwp3G</t>
+  </si>
+  <si>
+    <t>EKSA E900 Pro USB Gaming Headset for PC - Computer Headset with Detachable Noise Cancelling Mic, 7.1 Surround Sound, 50MM Driver - Headphones with Microphone for PS4/PS5, Xbox One, Laptop, Office</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4ufS1zS</t>
+  </si>
+  <si>
+    <t>HyperX Cloud III Wired Gaming Headset — Immersive DTS Spatial Audio, Powerful 53mm Drivers, Detachable Mic &amp; Signature HyperX Comfort for PC and Consoles</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4ok0cdd</t>
+  </si>
+  <si>
+    <t>Logitech G733 Lightspeed Wireless Gaming Headset, Suspension Headband, Lightsync RGB, Blue VO!CE Mic, PRO-G Audio – Black, Gaming Headset Wireless, PC, PS5, PS4, Switch Compatible</t>
+  </si>
+  <si>
+    <t>https://amzn.to/3S7ybcN</t>
+  </si>
+  <si>
+    <t>Wireless Gaming Headset for PC Over Ear Headphones with Mic Noise Cancelling Multi Platform Headset,7.1 Surround Sound,50mm Drivers,RGB,Aluminum Frame,Memory Foam Ear Pads for Xbox,PS5,Switch,Mobile</t>
+  </si>
+  <si>
+    <t>https://amzn.to/3S5Fce5</t>
+  </si>
+  <si>
+    <t>Razer Kraken V3 X Wired USB Gaming Headset: Lightweight Build - Triforce 40mm Drivers - HyperClear Cardioid Mic - 7.1 Surround Sound - Chroma RGB Lighting - Black</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4dRMeMd</t>
+  </si>
+  <si>
+    <t>KZ ZAR in-Ear Monitor 7BA+1DD Hybrid Drivers Gaming Earbuds HiFi Bass Noise Isolation IEM, Clarity in All Frequency Stereo Comfort-fit in Ear Headphones for Audio Engineers, Musicians(No Mic)</t>
+  </si>
+  <si>
+    <t>https://amzn.to/3RGyyLp</t>
+  </si>
+  <si>
+    <t>NUBWO HG03 Wired USB-A Gaming Headset for PC, Computer Headset with 7.1 Surround Sound, Noise Canceling Mic, 50MM Driver, Wired Headphones for PC, Laptop, Office - White</t>
+  </si>
+  <si>
+    <t>https://amzn.to/4e5RN8q</t>
   </si>
 </sst>
 </file>
@@ -550,7 +886,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -581,12 +917,14 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1549,49 +1887,49 @@
       <c r="B22" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="19" t="s">
+      <c r="C22" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="21">
         <v>249.99</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="E22" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="16"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
     </row>
     <row r="23" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A23" s="11"/>
       <c r="B23" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="C23" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="21">
         <v>228.89</v>
       </c>
-      <c r="E23" s="17" t="s">
+      <c r="E23" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="H23" s="16"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="16"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
     </row>
     <row r="24" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A24" s="11"/>
       <c r="B24" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="C24" s="22" t="s">
         <v>128</v>
       </c>
       <c r="D24" s="1">
         <v>124.99</v>
       </c>
-      <c r="E24" s="18" t="s">
+      <c r="E24" s="19" t="s">
         <v>129</v>
       </c>
     </row>
@@ -1600,13 +1938,13 @@
       <c r="B25" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="C25" s="22" t="s">
         <v>130</v>
       </c>
       <c r="D25" s="1">
         <v>169.99</v>
       </c>
-      <c r="E25" s="18" t="s">
+      <c r="E25" s="19" t="s">
         <v>131</v>
       </c>
     </row>
@@ -1615,13 +1953,13 @@
       <c r="B26" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C26" s="22" t="s">
         <v>132</v>
       </c>
       <c r="D26" s="1">
         <v>106.99</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="E26" s="19" t="s">
         <v>133</v>
       </c>
     </row>
@@ -1630,13 +1968,13 @@
       <c r="B27" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="C27" s="22" t="s">
         <v>134</v>
       </c>
       <c r="D27" s="1">
         <v>194.99</v>
       </c>
-      <c r="E27" s="18" t="s">
+      <c r="E27" s="19" t="s">
         <v>135</v>
       </c>
     </row>
@@ -1645,203 +1983,1103 @@
       <c r="B28" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C28" s="22" t="s">
         <v>136</v>
       </c>
       <c r="D28" s="1">
         <v>99.99</v>
       </c>
-      <c r="E28" s="18" t="s">
+      <c r="E28" s="19" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A29" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" s="14"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+    </row>
+    <row r="31" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B31" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="D31" s="17">
+        <v>99.99</v>
+      </c>
+      <c r="E31" s="19" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A32" s="11"/>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B32" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="D32" s="17">
+        <v>163.9</v>
+      </c>
+      <c r="E32" s="19" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A33" s="11"/>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B33" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="D33" s="17">
+        <v>389.99</v>
+      </c>
+      <c r="E33" s="19" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A34" s="11"/>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B34" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>145</v>
+      </c>
+      <c r="D34" s="17">
+        <v>89.99</v>
+      </c>
+      <c r="E34" s="19" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A35" s="11"/>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B35" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="D35" s="17">
+        <v>87.37</v>
+      </c>
+      <c r="E35" s="19" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A36" s="11"/>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B36" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="D36" s="17">
+        <v>299.95</v>
+      </c>
+      <c r="E36" s="19" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A37" s="11"/>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B37" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="D37" s="23">
+        <v>85.99</v>
+      </c>
+      <c r="E37" s="19" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="14"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="12"/>
+    </row>
+    <row r="40" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B40" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="D40">
+        <v>89.99</v>
+      </c>
+      <c r="E40" s="19" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A41" s="11"/>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B41" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="D41">
+        <v>99.99</v>
+      </c>
+      <c r="E41" s="19" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A42" s="11"/>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B42" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C42" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="D42">
+        <v>89.99</v>
+      </c>
+      <c r="E42" s="19" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A43" s="11"/>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B43" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="16" t="s">
+        <v>159</v>
+      </c>
+      <c r="D43">
+        <v>99.99</v>
+      </c>
+      <c r="E43" s="19" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A44" s="11"/>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B44" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C44" s="16" t="s">
+        <v>161</v>
+      </c>
+      <c r="D44">
+        <v>79.989999999999995</v>
+      </c>
+      <c r="E44" s="19" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A45" s="11"/>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B45" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D45">
+        <v>49.99</v>
+      </c>
+      <c r="E45" s="19" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A46" s="11"/>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B46" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C46" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="D46">
+        <v>64.989999999999995</v>
+      </c>
+      <c r="E46" s="19" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E47" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="14"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="12"/>
+      <c r="D48" s="12"/>
+      <c r="E48" s="12"/>
+    </row>
+    <row r="49" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A49" s="11" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B49" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C49" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="D49">
+        <v>92.99</v>
+      </c>
+      <c r="E49" s="19" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A50" s="11"/>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B50" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C50" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="D50">
+        <v>96.99</v>
+      </c>
+      <c r="E50" s="19" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A51" s="11"/>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B51" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C51" s="16" t="s">
+        <v>171</v>
+      </c>
+      <c r="D51">
+        <v>83.99</v>
+      </c>
+      <c r="E51" s="19" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A52" s="11"/>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B52" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="D52">
+        <v>129.99</v>
+      </c>
+      <c r="E52" s="19" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A53" s="11"/>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B53" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C53" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="D53">
+        <v>52.99</v>
+      </c>
+      <c r="E53" s="19" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A54" s="11"/>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B54" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C54" s="16" t="s">
+        <v>177</v>
+      </c>
+      <c r="D54">
+        <v>49.99</v>
+      </c>
+      <c r="E54" s="19" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A55" s="11"/>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B55" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C55" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="D55">
+        <v>44.9</v>
+      </c>
+      <c r="E55" s="19" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B56" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D56" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E56" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="14"/>
+      <c r="B57" s="15"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="12"/>
+    </row>
+    <row r="58" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A58" s="11" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B58" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C58" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="D58">
+        <v>57.69</v>
+      </c>
+      <c r="E58" s="19" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A59" s="11"/>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B59" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C59" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="D59">
+        <v>22.9</v>
+      </c>
+      <c r="E59" s="19" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A60" s="11"/>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B60" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C60" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="D60">
+        <v>25.99</v>
+      </c>
+      <c r="E60" s="19" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A61" s="11"/>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B61" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="D61">
+        <v>164.95</v>
+      </c>
+      <c r="E61" s="19" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A62" s="11"/>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B62" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C62" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="D62">
+        <v>34.9</v>
+      </c>
+      <c r="E62" s="19" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A63" s="11"/>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B63" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C63" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="D63">
+        <v>49.99</v>
+      </c>
+      <c r="E63" s="19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A64" s="11"/>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B64" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C64" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="D64">
+        <v>33.9</v>
+      </c>
+      <c r="E64" s="19" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B65" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C65" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D65" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E65" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="14"/>
+      <c r="B66" s="15"/>
+      <c r="C66" s="12"/>
+      <c r="D66" s="12"/>
+      <c r="E66" s="12"/>
+    </row>
+    <row r="67" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A67" s="11" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B67" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C67" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="D67">
+        <v>69.989999999999995</v>
+      </c>
+      <c r="E67" s="19" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A68" s="11"/>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B68" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C68" s="16" t="s">
+        <v>197</v>
+      </c>
+      <c r="D68">
+        <v>79.989999999999995</v>
+      </c>
+      <c r="E68" s="19" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A69" s="11"/>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B69" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C69" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="D69">
+        <v>86.99</v>
+      </c>
+      <c r="E69" s="19" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A70" s="11"/>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B70" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="D70">
+        <v>169</v>
+      </c>
+      <c r="E70" s="19" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A71" s="11"/>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B71" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C71" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="D71">
+        <v>89.99</v>
+      </c>
+      <c r="E71" s="19" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A72" s="11"/>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B72" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C72" s="16" t="s">
+        <v>205</v>
+      </c>
+      <c r="D72">
+        <v>89.99</v>
+      </c>
+      <c r="E72" s="19" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A73" s="11"/>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B73" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C73" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="D73">
+        <v>79.989999999999995</v>
+      </c>
+      <c r="E73" s="19" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B74" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C74" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D74" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E74" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="14"/>
+      <c r="B75" s="15"/>
+      <c r="C75" s="12"/>
+      <c r="D75" s="12"/>
+      <c r="E75" s="12"/>
+    </row>
+    <row r="76" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A76" s="11" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B76" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C76" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="D76">
+        <v>39.99</v>
+      </c>
+      <c r="E76" s="19" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A77" s="11"/>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B77" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C77" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="D77">
+        <v>68.989999999999995</v>
+      </c>
+      <c r="E77" s="19" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A78" s="11"/>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B78" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C78" s="16" t="s">
+        <v>213</v>
+      </c>
+      <c r="D78">
+        <v>65.540000000000006</v>
+      </c>
+      <c r="E78" s="19" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A79" s="11"/>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B79" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C79" s="16" t="s">
+        <v>215</v>
+      </c>
+      <c r="D79">
+        <v>29.99</v>
+      </c>
+      <c r="E79" s="19" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A80" s="11"/>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B80" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C80" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="D80">
+        <v>69.989999999999995</v>
+      </c>
+      <c r="E80" s="19" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A81" s="11"/>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B81" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C81" s="16" t="s">
+        <v>219</v>
+      </c>
+      <c r="D81">
+        <v>53.99</v>
+      </c>
+      <c r="E81" s="19" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A82" s="11"/>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B82" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C82" s="16" t="s">
+        <v>221</v>
+      </c>
+      <c r="D82">
+        <v>71.989999999999995</v>
+      </c>
+      <c r="E82" s="19" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B83" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C83" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D83" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E83" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="14"/>
+      <c r="B84" s="15"/>
+      <c r="C84" s="12"/>
+      <c r="D84" s="12"/>
+      <c r="E84" s="12"/>
+    </row>
+    <row r="85" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A85" s="11" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B85" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C85" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="D85">
+        <v>37.71</v>
+      </c>
+      <c r="E85" s="19" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A86" s="11"/>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B86" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C86" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="D86">
+        <v>129.94999999999999</v>
+      </c>
+      <c r="E86" s="19" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A87" s="11"/>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B87" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C87" s="16" t="s">
+        <v>227</v>
+      </c>
+      <c r="D87">
+        <v>37.99</v>
+      </c>
+      <c r="E87" s="19" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A88" s="11"/>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B88" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C88" s="16" t="s">
+        <v>229</v>
+      </c>
+      <c r="D88">
+        <v>159.99</v>
+      </c>
+      <c r="E88" s="19" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A89" s="11"/>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B89" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C89" s="16" t="s">
+        <v>231</v>
+      </c>
+      <c r="D89">
+        <v>79.95</v>
+      </c>
+      <c r="E89" s="19" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A90" s="11"/>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B90" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C90" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="D90">
+        <v>42.99</v>
+      </c>
+      <c r="E90" s="19" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A91" s="11"/>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B91" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C91" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="D91">
+        <v>48.99</v>
+      </c>
+      <c r="E91" s="19" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B92" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C92" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D92" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E92" s="12" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A93" s="14"/>
+      <c r="B93" s="15"/>
+      <c r="C93" s="12"/>
+      <c r="D93" s="12"/>
+      <c r="E93" s="12"/>
+    </row>
+    <row r="94" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A94" s="11" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B94" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C94" s="16" t="s">
+        <v>237</v>
+      </c>
+      <c r="D94">
+        <v>49.99</v>
+      </c>
+      <c r="E94" s="19" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A95" s="11"/>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B95" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C95" s="16" t="s">
+        <v>239</v>
+      </c>
+      <c r="D95">
+        <v>57.99</v>
+      </c>
+      <c r="E95" s="19" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A96" s="11"/>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B96" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C96" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="D96">
+        <v>128.99</v>
+      </c>
+      <c r="E96" s="19" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A97" s="11"/>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B97" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C97" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="D97">
+        <v>89.99</v>
+      </c>
+      <c r="E97" s="19" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A98" s="11"/>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B98" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C98" s="16" t="s">
+        <v>245</v>
+      </c>
+      <c r="D98">
+        <v>39.979999999999997</v>
+      </c>
+      <c r="E98" s="19" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A99" s="11"/>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B99" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C99" s="16" t="s">
+        <v>247</v>
+      </c>
+      <c r="D99">
+        <v>99.99</v>
+      </c>
+      <c r="E99" s="19" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A100" s="11"/>
+      <c r="B100" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C100" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="D100">
+        <v>35.99</v>
+      </c>
+      <c r="E100" s="19" t="s">
+        <v>250</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="46">
+  <mergeCells count="86">
+    <mergeCell ref="B92:B93"/>
+    <mergeCell ref="C92:C93"/>
+    <mergeCell ref="D92:D93"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="E74:E75"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="E92:E93"/>
+    <mergeCell ref="B74:B75"/>
+    <mergeCell ref="C74:C75"/>
+    <mergeCell ref="D74:D75"/>
+    <mergeCell ref="A83:A84"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="C83:C84"/>
+    <mergeCell ref="D83:D84"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="D65:D66"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="D47:D48"/>
     <mergeCell ref="L20:L21"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="E29:E30"/>
     <mergeCell ref="G20:G21"/>
     <mergeCell ref="H20:H21"/>
     <mergeCell ref="I20:I21"/>
@@ -1887,6 +3125,10 @@
     <mergeCell ref="A49:A55"/>
     <mergeCell ref="A58:A64"/>
     <mergeCell ref="A67:A73"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="A56:A57"/>
+    <mergeCell ref="A74:A75"/>
+    <mergeCell ref="A92:A93"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -1911,8 +3153,64 @@
     <hyperlink ref="E26" r:id="rId19" xr:uid="{1A3E1B3E-7A6D-4A7F-B66D-79C359972A55}"/>
     <hyperlink ref="E27" r:id="rId20" xr:uid="{25AD8478-EB11-46A4-B6A0-480D08954434}"/>
     <hyperlink ref="E28" r:id="rId21" xr:uid="{D5D911D0-2140-44B2-9188-B2BDD62FF360}"/>
+    <hyperlink ref="E31" r:id="rId22" xr:uid="{503CC57F-3B31-4190-B6E3-6B892A8A31CB}"/>
+    <hyperlink ref="E32" r:id="rId23" xr:uid="{DF2EDB3C-3149-4A72-9F0E-37D34E68700E}"/>
+    <hyperlink ref="E33" r:id="rId24" xr:uid="{F99EB831-10FB-480E-9981-8A80708A5F48}"/>
+    <hyperlink ref="E34" r:id="rId25" xr:uid="{56980B0F-9AD2-4095-8352-CCB15AC9D66C}"/>
+    <hyperlink ref="E35" r:id="rId26" xr:uid="{C9788AE7-8329-4E9F-94CA-55AE43EC56CD}"/>
+    <hyperlink ref="E36" r:id="rId27" xr:uid="{E7902C2B-A4DD-48DB-9DF0-6117EE85B97C}"/>
+    <hyperlink ref="E37" r:id="rId28" xr:uid="{925F456E-3436-4115-9879-F7C2A44D6ABD}"/>
+    <hyperlink ref="E40" r:id="rId29" xr:uid="{390457BD-E67E-4C43-8DD1-7B6F9DFC8DC4}"/>
+    <hyperlink ref="E41" r:id="rId30" xr:uid="{68502FCC-D77B-41D7-A25C-5DBAC5817742}"/>
+    <hyperlink ref="E42" r:id="rId31" xr:uid="{E4BC909E-B7BB-46A6-852B-0ED96D7BCE60}"/>
+    <hyperlink ref="E43" r:id="rId32" xr:uid="{AB00DDA6-5807-4394-B6BA-D28E79E01505}"/>
+    <hyperlink ref="E44" r:id="rId33" xr:uid="{DF09E5B9-CB1A-466D-93DA-A97DD1EF30C5}"/>
+    <hyperlink ref="E45" r:id="rId34" xr:uid="{B15E1696-4580-4848-8FF7-064BAA87C68E}"/>
+    <hyperlink ref="E46" r:id="rId35" xr:uid="{EA8992CE-5BE5-427D-97DA-000BDE8BD4CE}"/>
+    <hyperlink ref="E49" r:id="rId36" xr:uid="{90662FEC-566E-4E01-9F9C-891C89141AE0}"/>
+    <hyperlink ref="E50" r:id="rId37" xr:uid="{4DA2B167-CD3E-408C-8B65-B81E9206F0FD}"/>
+    <hyperlink ref="E51" r:id="rId38" xr:uid="{C7EDC0A9-A5B8-4390-AA97-9E030E0B526C}"/>
+    <hyperlink ref="E52" r:id="rId39" xr:uid="{8BDEE4A2-5D93-46B0-8E10-45B1E154B190}"/>
+    <hyperlink ref="E53" r:id="rId40" xr:uid="{1CB05ADD-99F1-44C4-A596-C2DE02632F97}"/>
+    <hyperlink ref="E54" r:id="rId41" xr:uid="{42CAD64A-9570-4C1F-857F-C22F5C92E169}"/>
+    <hyperlink ref="E55" r:id="rId42" xr:uid="{DF02251D-684A-4BF7-9859-A6154F69A1E6}"/>
+    <hyperlink ref="E58" r:id="rId43" xr:uid="{950E3EF0-44FA-4EB0-9A24-51BE86D5F738}"/>
+    <hyperlink ref="E59" r:id="rId44" xr:uid="{13F7BC4B-9AE9-4C8B-AF86-8687A03D4F7E}"/>
+    <hyperlink ref="E60" r:id="rId45" xr:uid="{5893B067-413F-4279-B0BC-40AB299BE549}"/>
+    <hyperlink ref="E61" r:id="rId46" xr:uid="{46146695-697F-46DD-A65A-8B046612A307}"/>
+    <hyperlink ref="E62" r:id="rId47" xr:uid="{2834BA6C-4A20-4423-9126-94FE22C63D6B}"/>
+    <hyperlink ref="E63" r:id="rId48" xr:uid="{1C80F072-F644-4639-9128-504D73A89463}"/>
+    <hyperlink ref="E67" r:id="rId49" xr:uid="{BFE0785F-4BAE-452C-83D8-38D16059614E}"/>
+    <hyperlink ref="E68" r:id="rId50" xr:uid="{74E0B19C-3F5D-458D-863F-4503F98442CA}"/>
+    <hyperlink ref="E69" r:id="rId51" xr:uid="{6B447A40-7470-4191-A25B-061771FEA0DF}"/>
+    <hyperlink ref="E70" r:id="rId52" xr:uid="{34616ED8-0497-473A-B3BF-1EBAC5B4DD27}"/>
+    <hyperlink ref="E71" r:id="rId53" xr:uid="{D45BC6B6-918D-4876-AD5A-BA57DBB79EE6}"/>
+    <hyperlink ref="E72" r:id="rId54" xr:uid="{E35618C1-59D6-4192-87C8-ECC90AB8BF08}"/>
+    <hyperlink ref="E73" r:id="rId55" xr:uid="{AFCA5929-B25B-43B1-87A6-4DD2FCAE81CC}"/>
+    <hyperlink ref="E76" r:id="rId56" xr:uid="{8CD3ED2D-6BF8-4476-AC19-F886DA23C0D5}"/>
+    <hyperlink ref="E77" r:id="rId57" xr:uid="{160495B7-B7BB-43FC-AC9C-01C0C367F765}"/>
+    <hyperlink ref="E78" r:id="rId58" xr:uid="{60C1B31C-F8FB-4787-9FAB-376AFE78FCDB}"/>
+    <hyperlink ref="E79" r:id="rId59" xr:uid="{9F6C663B-F6C7-4790-B5B8-4CA36E209011}"/>
+    <hyperlink ref="E80" r:id="rId60" xr:uid="{B39CFDD8-3D9F-4952-9A3F-55D4D7BABF63}"/>
+    <hyperlink ref="E81" r:id="rId61" xr:uid="{F0E81686-D10C-4D19-8110-FD92170B3EF0}"/>
+    <hyperlink ref="E82" r:id="rId62" xr:uid="{8A0A49F5-A968-4C25-A15B-A933DBFDD107}"/>
+    <hyperlink ref="E85" r:id="rId63" xr:uid="{2C847E71-9A42-4BEC-811F-9B68942FDB2A}"/>
+    <hyperlink ref="E86" r:id="rId64" xr:uid="{05DB885B-60C5-4484-B49E-9D1E0021096E}"/>
+    <hyperlink ref="E87" r:id="rId65" xr:uid="{346B4A18-B949-4127-9317-91AAC9D730AC}"/>
+    <hyperlink ref="E88" r:id="rId66" xr:uid="{D2549A2F-02E8-4386-9544-D64A6B058981}"/>
+    <hyperlink ref="E89" r:id="rId67" xr:uid="{B7507357-0768-40B3-BF94-9D3712868545}"/>
+    <hyperlink ref="E90" r:id="rId68" xr:uid="{31BE5BB4-4B2F-4BC7-8677-0F0EBB68DB74}"/>
+    <hyperlink ref="E91" r:id="rId69" xr:uid="{C4782FB5-2464-4FF2-A7E6-7D07CBDF2D8E}"/>
+    <hyperlink ref="E64" r:id="rId70" xr:uid="{07099841-3D49-4748-8F82-6FE49B0F17EF}"/>
+    <hyperlink ref="E94" r:id="rId71" xr:uid="{6578CB3D-62AD-4DA5-A227-7CD66E43C0BE}"/>
+    <hyperlink ref="E95" r:id="rId72" xr:uid="{06D41B9C-7C7E-45A7-A27C-BBC5BBC022F4}"/>
+    <hyperlink ref="E96" r:id="rId73" xr:uid="{BEF22BCA-D151-4667-AF57-FD2D63CC10C9}"/>
+    <hyperlink ref="E97" r:id="rId74" xr:uid="{2888B9BA-783B-470D-B85B-FC84ABDD1FDF}"/>
+    <hyperlink ref="E98" r:id="rId75" xr:uid="{F5BBD7AF-735A-443C-A91D-0D1978380837}"/>
+    <hyperlink ref="E99" r:id="rId76" xr:uid="{E766F4BB-121D-4899-8F2C-08102F7920B1}"/>
+    <hyperlink ref="E100" r:id="rId77" xr:uid="{69116B45-E7F9-4D91-8610-9198BFA38371}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId22"/>
+  <pageSetup orientation="portrait" r:id="rId78"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
se suben todas las imagenes de los primeros 4 componentes
</commit_message>
<xml_diff>
--- a/Products.xlsx
+++ b/Products.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyecto Astro\zona-gaming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B3B3673-1D0F-4B7B-B6A8-28C405626EDD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E779EA69-0692-42CF-86C6-398397C8418F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32520" yWindow="2070" windowWidth="20115" windowHeight="11340" xr2:uid="{0CBE72FF-69DA-4304-99BE-1A2A53C4AD2D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0CBE72FF-69DA-4304-99BE-1A2A53C4AD2D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
se suben el resto de imagenes
</commit_message>
<xml_diff>
--- a/Products.xlsx
+++ b/Products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyecto Astro\zona-gaming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E779EA69-0692-42CF-86C6-398397C8418F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013519D2-1CD5-4324-9670-B7C7C07FA205}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0CBE72FF-69DA-4304-99BE-1A2A53C4AD2D}"/>
   </bookViews>
@@ -886,7 +886,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -902,29 +902,31 @@
     <xf numFmtId="8" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1256,55 +1258,55 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="K2" s="19" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="14"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="12"/>
+      <c r="A3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="19"/>
     </row>
     <row r="4" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -1339,7 +1341,7 @@
       </c>
     </row>
     <row r="5" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="11"/>
+      <c r="A5" s="22"/>
       <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
@@ -1372,11 +1374,11 @@
       </c>
     </row>
     <row r="6" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="11"/>
+      <c r="A6" s="22"/>
       <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="14" t="s">
         <v>35</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -1405,7 +1407,7 @@
       </c>
     </row>
     <row r="7" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A7" s="11"/>
+      <c r="A7" s="22"/>
       <c r="B7" s="3" t="s">
         <v>4</v>
       </c>
@@ -1438,7 +1440,7 @@
       </c>
     </row>
     <row r="8" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A8" s="11"/>
+      <c r="A8" s="22"/>
       <c r="B8" s="3" t="s">
         <v>5</v>
       </c>
@@ -1471,11 +1473,11 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A9" s="11"/>
+      <c r="A9" s="22"/>
       <c r="B9" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="14" t="s">
         <v>57</v>
       </c>
       <c r="D9" s="2" t="s">
@@ -1504,7 +1506,7 @@
       </c>
     </row>
     <row r="10" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="11"/>
+      <c r="A10" s="22"/>
       <c r="B10" s="3" t="s">
         <v>7</v>
       </c>
@@ -1537,59 +1539,59 @@
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="G11" s="12" t="s">
+      <c r="G11" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="I11" s="12" t="s">
+      <c r="I11" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="J11" s="12" t="s">
+      <c r="J11" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="K11" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="L11" s="12" t="s">
+      <c r="L11" s="19" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="13"/>
-      <c r="L12" s="12"/>
+      <c r="A12" s="20"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="21"/>
+      <c r="L12" s="19"/>
     </row>
     <row r="13" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="22" t="s">
         <v>17</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -1622,12 +1624,12 @@
       <c r="K13" s="8">
         <v>179</v>
       </c>
-      <c r="L13" s="4" t="s">
+      <c r="L13" s="23" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A14" s="11"/>
+      <c r="A14" s="22"/>
       <c r="B14" s="3" t="s">
         <v>2</v>
       </c>
@@ -1658,12 +1660,12 @@
       <c r="K14" s="8">
         <v>315</v>
       </c>
-      <c r="L14" s="4" t="s">
+      <c r="L14" s="23" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A15" s="11"/>
+      <c r="A15" s="22"/>
       <c r="B15" s="3" t="s">
         <v>3</v>
       </c>
@@ -1694,12 +1696,12 @@
       <c r="K15" s="8">
         <v>84</v>
       </c>
-      <c r="L15" s="4" t="s">
+      <c r="L15" s="23" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A16" s="11"/>
+      <c r="A16" s="22"/>
       <c r="B16" s="3" t="s">
         <v>4</v>
       </c>
@@ -1730,12 +1732,12 @@
       <c r="K16" s="8">
         <v>227.45</v>
       </c>
-      <c r="L16" s="4" t="s">
+      <c r="L16" s="23" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A17" s="11"/>
+      <c r="A17" s="22"/>
       <c r="B17" s="3" t="s">
         <v>5</v>
       </c>
@@ -1766,12 +1768,12 @@
       <c r="K17" s="8">
         <v>167</v>
       </c>
-      <c r="L17" s="4" t="s">
+      <c r="L17" s="23" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A18" s="11"/>
+      <c r="A18" s="22"/>
       <c r="B18" s="3" t="s">
         <v>6</v>
       </c>
@@ -1802,12 +1804,12 @@
       <c r="K18" s="8">
         <v>234</v>
       </c>
-      <c r="L18" s="4" t="s">
+      <c r="L18" s="23" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A19" s="11"/>
+      <c r="A19" s="22"/>
       <c r="B19" s="3" t="s">
         <v>7</v>
       </c>
@@ -1838,1253 +1840,1238 @@
       <c r="K19" s="8">
         <v>218.98</v>
       </c>
-      <c r="L19" s="4" t="s">
+      <c r="L19" s="23" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="19" t="s">
         <v>138</v>
       </c>
-      <c r="F20" s="13"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="13"/>
-      <c r="L20" s="12"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="21"/>
+      <c r="L20" s="19"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21" s="14"/>
-      <c r="B21" s="15"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="12"/>
-      <c r="J21" s="12"/>
-      <c r="K21" s="13"/>
-      <c r="L21" s="12"/>
+      <c r="A21" s="20"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="21"/>
+      <c r="I21" s="19"/>
+      <c r="J21" s="19"/>
+      <c r="K21" s="21"/>
+      <c r="L21" s="19"/>
     </row>
     <row r="22" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="22" t="s">
         <v>115</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="C22" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="D22" s="21">
+      <c r="D22" s="15">
         <v>249.99</v>
       </c>
-      <c r="E22" s="18" t="s">
+      <c r="E22" s="24" t="s">
         <v>127</v>
       </c>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="17"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
     </row>
     <row r="23" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A23" s="11"/>
+      <c r="A23" s="22"/>
       <c r="B23" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C23" s="22" t="s">
+      <c r="C23" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="D23" s="21">
+      <c r="D23" s="15">
         <v>228.89</v>
       </c>
-      <c r="E23" s="18" t="s">
+      <c r="E23" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
     </row>
     <row r="24" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A24" s="11"/>
+      <c r="A24" s="22"/>
       <c r="B24" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="C24" s="16" t="s">
         <v>128</v>
       </c>
       <c r="D24" s="1">
         <v>124.99</v>
       </c>
-      <c r="E24" s="19" t="s">
+      <c r="E24" s="25" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A25" s="11"/>
+      <c r="A25" s="22"/>
       <c r="B25" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C25" s="22" t="s">
+      <c r="C25" s="16" t="s">
         <v>130</v>
       </c>
       <c r="D25" s="1">
         <v>169.99</v>
       </c>
-      <c r="E25" s="19" t="s">
+      <c r="E25" s="25" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A26" s="11"/>
+      <c r="A26" s="22"/>
       <c r="B26" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="C26" s="16" t="s">
         <v>132</v>
       </c>
       <c r="D26" s="1">
         <v>106.99</v>
       </c>
-      <c r="E26" s="19" t="s">
+      <c r="E26" s="25" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A27" s="11"/>
+      <c r="A27" s="22"/>
       <c r="B27" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C27" s="22" t="s">
+      <c r="C27" s="16" t="s">
         <v>134</v>
       </c>
       <c r="D27" s="1">
         <v>194.99</v>
       </c>
-      <c r="E27" s="19" t="s">
+      <c r="E27" s="25" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A28" s="11"/>
+      <c r="A28" s="22"/>
       <c r="B28" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="16" t="s">
         <v>136</v>
       </c>
       <c r="D28" s="1">
         <v>99.99</v>
       </c>
-      <c r="E28" s="19" t="s">
+      <c r="E28" s="25" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B29" s="15" t="s">
+      <c r="B29" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="C29" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D29" s="12" t="s">
+      <c r="D29" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="E29" s="12" t="s">
+      <c r="E29" s="19" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A30" s="14"/>
-      <c r="B30" s="15"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="18"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
     </row>
     <row r="31" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="22" t="s">
         <v>116</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="16" t="s">
+      <c r="C31" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="D31" s="17">
+      <c r="D31" s="12">
         <v>99.99</v>
       </c>
-      <c r="E31" s="19" t="s">
+      <c r="E31" s="25" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="32" spans="1:12" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A32" s="11"/>
+      <c r="A32" s="22"/>
       <c r="B32" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C32" s="16" t="s">
+      <c r="C32" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="D32" s="17">
+      <c r="D32" s="12">
         <v>163.9</v>
       </c>
-      <c r="E32" s="19" t="s">
+      <c r="E32" s="25" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A33" s="11"/>
+      <c r="A33" s="22"/>
       <c r="B33" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C33" s="16" t="s">
+      <c r="C33" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="D33" s="17">
+      <c r="D33" s="12">
         <v>389.99</v>
       </c>
-      <c r="E33" s="19" t="s">
+      <c r="E33" s="25" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A34" s="11"/>
+      <c r="A34" s="22"/>
       <c r="B34" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C34" s="16" t="s">
+      <c r="C34" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="D34" s="17">
+      <c r="D34" s="12">
         <v>89.99</v>
       </c>
-      <c r="E34" s="19" t="s">
+      <c r="E34" s="25" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A35" s="11"/>
+      <c r="A35" s="22"/>
       <c r="B35" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C35" s="16" t="s">
+      <c r="C35" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="D35" s="17">
+      <c r="D35" s="12">
         <v>87.37</v>
       </c>
-      <c r="E35" s="19" t="s">
+      <c r="E35" s="25" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A36" s="11"/>
+      <c r="A36" s="22"/>
       <c r="B36" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C36" s="16" t="s">
+      <c r="C36" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="D36" s="17">
+      <c r="D36" s="12">
         <v>299.95</v>
       </c>
-      <c r="E36" s="19" t="s">
+      <c r="E36" s="25" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A37" s="11"/>
+      <c r="A37" s="22"/>
       <c r="B37" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C37" s="16" t="s">
+      <c r="C37" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="D37" s="23">
+      <c r="D37" s="17">
         <v>85.99</v>
       </c>
-      <c r="E37" s="19" t="s">
+      <c r="E37" s="25" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="14" t="s">
+      <c r="A38" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B38" s="15" t="s">
+      <c r="B38" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C38" s="12" t="s">
+      <c r="C38" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D38" s="12" t="s">
+      <c r="D38" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="E38" s="12" t="s">
+      <c r="E38" s="19" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="14"/>
-      <c r="B39" s="15"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="12"/>
+      <c r="A39" s="20"/>
+      <c r="B39" s="18"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="19"/>
     </row>
     <row r="40" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A40" s="11" t="s">
+      <c r="A40" s="22" t="s">
         <v>117</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C40" s="16" t="s">
+      <c r="C40" s="11" t="s">
         <v>153</v>
       </c>
       <c r="D40">
         <v>89.99</v>
       </c>
-      <c r="E40" s="19" t="s">
+      <c r="E40" s="25" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A41" s="11"/>
+      <c r="A41" s="22"/>
       <c r="B41" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C41" s="16" t="s">
+      <c r="C41" s="11" t="s">
         <v>155</v>
       </c>
       <c r="D41">
         <v>99.99</v>
       </c>
-      <c r="E41" s="19" t="s">
+      <c r="E41" s="25" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A42" s="11"/>
+      <c r="A42" s="22"/>
       <c r="B42" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C42" s="16" t="s">
+      <c r="C42" s="11" t="s">
         <v>157</v>
       </c>
       <c r="D42">
         <v>89.99</v>
       </c>
-      <c r="E42" s="19" t="s">
+      <c r="E42" s="25" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A43" s="11"/>
+      <c r="A43" s="22"/>
       <c r="B43" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C43" s="16" t="s">
+      <c r="C43" s="11" t="s">
         <v>159</v>
       </c>
       <c r="D43">
         <v>99.99</v>
       </c>
-      <c r="E43" s="19" t="s">
+      <c r="E43" s="25" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A44" s="11"/>
+      <c r="A44" s="22"/>
       <c r="B44" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C44" s="16" t="s">
+      <c r="C44" s="11" t="s">
         <v>161</v>
       </c>
       <c r="D44">
         <v>79.989999999999995</v>
       </c>
-      <c r="E44" s="19" t="s">
+      <c r="E44" s="25" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A45" s="11"/>
+      <c r="A45" s="22"/>
       <c r="B45" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C45" s="16" t="s">
+      <c r="C45" s="11" t="s">
         <v>163</v>
       </c>
       <c r="D45">
         <v>49.99</v>
       </c>
-      <c r="E45" s="19" t="s">
+      <c r="E45" s="25" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A46" s="11"/>
+      <c r="A46" s="22"/>
       <c r="B46" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="16" t="s">
+      <c r="C46" s="11" t="s">
         <v>165</v>
       </c>
       <c r="D46">
         <v>64.989999999999995</v>
       </c>
-      <c r="E46" s="19" t="s">
+      <c r="E46" s="25" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="14" t="s">
+      <c r="A47" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="B47" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C47" s="12" t="s">
+      <c r="C47" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D47" s="12" t="s">
+      <c r="D47" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="E47" s="12" t="s">
+      <c r="E47" s="19" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="14"/>
-      <c r="B48" s="15"/>
-      <c r="C48" s="12"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="12"/>
+      <c r="A48" s="20"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="19"/>
     </row>
     <row r="49" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A49" s="11" t="s">
+      <c r="A49" s="22" t="s">
         <v>118</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C49" s="16" t="s">
+      <c r="C49" s="11" t="s">
         <v>167</v>
       </c>
       <c r="D49">
         <v>92.99</v>
       </c>
-      <c r="E49" s="19" t="s">
+      <c r="E49" s="25" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A50" s="11"/>
+      <c r="A50" s="22"/>
       <c r="B50" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C50" s="16" t="s">
+      <c r="C50" s="11" t="s">
         <v>169</v>
       </c>
       <c r="D50">
         <v>96.99</v>
       </c>
-      <c r="E50" s="19" t="s">
+      <c r="E50" s="25" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A51" s="11"/>
+      <c r="A51" s="22"/>
       <c r="B51" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C51" s="16" t="s">
+      <c r="C51" s="11" t="s">
         <v>171</v>
       </c>
       <c r="D51">
         <v>83.99</v>
       </c>
-      <c r="E51" s="19" t="s">
+      <c r="E51" s="25" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A52" s="11"/>
+      <c r="A52" s="22"/>
       <c r="B52" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C52" s="16" t="s">
+      <c r="C52" s="11" t="s">
         <v>173</v>
       </c>
       <c r="D52">
         <v>129.99</v>
       </c>
-      <c r="E52" s="19" t="s">
+      <c r="E52" s="25" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A53" s="11"/>
+      <c r="A53" s="22"/>
       <c r="B53" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C53" s="16" t="s">
+      <c r="C53" s="11" t="s">
         <v>175</v>
       </c>
       <c r="D53">
         <v>52.99</v>
       </c>
-      <c r="E53" s="19" t="s">
+      <c r="E53" s="25" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A54" s="11"/>
+      <c r="A54" s="22"/>
       <c r="B54" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C54" s="16" t="s">
+      <c r="C54" s="11" t="s">
         <v>177</v>
       </c>
       <c r="D54">
         <v>49.99</v>
       </c>
-      <c r="E54" s="19" t="s">
+      <c r="E54" s="25" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A55" s="11"/>
+      <c r="A55" s="22"/>
       <c r="B55" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C55" s="16" t="s">
+      <c r="C55" s="11" t="s">
         <v>179</v>
       </c>
       <c r="D55">
         <v>44.9</v>
       </c>
-      <c r="E55" s="19" t="s">
+      <c r="E55" s="25" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="14" t="s">
+      <c r="A56" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B56" s="15" t="s">
+      <c r="B56" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C56" s="12" t="s">
+      <c r="C56" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D56" s="12" t="s">
+      <c r="D56" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="E56" s="12" t="s">
+      <c r="E56" s="19" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="14"/>
-      <c r="B57" s="15"/>
-      <c r="C57" s="12"/>
-      <c r="D57" s="12"/>
-      <c r="E57" s="12"/>
+      <c r="A57" s="20"/>
+      <c r="B57" s="18"/>
+      <c r="C57" s="19"/>
+      <c r="D57" s="19"/>
+      <c r="E57" s="19"/>
     </row>
     <row r="58" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A58" s="11" t="s">
+      <c r="A58" s="22" t="s">
         <v>119</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C58" s="16" t="s">
+      <c r="C58" s="11" t="s">
         <v>181</v>
       </c>
       <c r="D58">
         <v>57.69</v>
       </c>
-      <c r="E58" s="19" t="s">
+      <c r="E58" s="13" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A59" s="11"/>
+      <c r="A59" s="22"/>
       <c r="B59" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C59" s="16" t="s">
+      <c r="C59" s="11" t="s">
         <v>183</v>
       </c>
       <c r="D59">
         <v>22.9</v>
       </c>
-      <c r="E59" s="19" t="s">
+      <c r="E59" s="13" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A60" s="11"/>
+      <c r="A60" s="22"/>
       <c r="B60" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C60" s="16" t="s">
+      <c r="C60" s="11" t="s">
         <v>185</v>
       </c>
       <c r="D60">
         <v>25.99</v>
       </c>
-      <c r="E60" s="19" t="s">
+      <c r="E60" s="13" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A61" s="11"/>
+      <c r="A61" s="22"/>
       <c r="B61" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C61" s="16" t="s">
+      <c r="C61" s="11" t="s">
         <v>187</v>
       </c>
       <c r="D61">
         <v>164.95</v>
       </c>
-      <c r="E61" s="19" t="s">
+      <c r="E61" s="13" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A62" s="11"/>
+      <c r="A62" s="22"/>
       <c r="B62" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C62" s="16" t="s">
+      <c r="C62" s="11" t="s">
         <v>189</v>
       </c>
       <c r="D62">
         <v>34.9</v>
       </c>
-      <c r="E62" s="19" t="s">
+      <c r="E62" s="13" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A63" s="11"/>
+      <c r="A63" s="22"/>
       <c r="B63" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C63" s="16" t="s">
+      <c r="C63" s="11" t="s">
         <v>191</v>
       </c>
       <c r="D63">
         <v>49.99</v>
       </c>
-      <c r="E63" s="19" t="s">
+      <c r="E63" s="13" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A64" s="11"/>
+      <c r="A64" s="22"/>
       <c r="B64" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C64" s="16" t="s">
+      <c r="C64" s="11" t="s">
         <v>193</v>
       </c>
       <c r="D64">
         <v>33.9</v>
       </c>
-      <c r="E64" s="19" t="s">
+      <c r="E64" s="13" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="14" t="s">
+      <c r="A65" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B65" s="15" t="s">
+      <c r="B65" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C65" s="12" t="s">
+      <c r="C65" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D65" s="12" t="s">
+      <c r="D65" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="E65" s="12" t="s">
+      <c r="E65" s="19" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="14"/>
-      <c r="B66" s="15"/>
-      <c r="C66" s="12"/>
-      <c r="D66" s="12"/>
-      <c r="E66" s="12"/>
+      <c r="A66" s="20"/>
+      <c r="B66" s="18"/>
+      <c r="C66" s="19"/>
+      <c r="D66" s="19"/>
+      <c r="E66" s="19"/>
     </row>
     <row r="67" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A67" s="11" t="s">
+      <c r="A67" s="22" t="s">
         <v>120</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C67" s="16" t="s">
+      <c r="C67" s="11" t="s">
         <v>195</v>
       </c>
       <c r="D67">
         <v>69.989999999999995</v>
       </c>
-      <c r="E67" s="19" t="s">
+      <c r="E67" s="13" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A68" s="11"/>
+      <c r="A68" s="22"/>
       <c r="B68" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C68" s="16" t="s">
+      <c r="C68" s="11" t="s">
         <v>197</v>
       </c>
       <c r="D68">
         <v>79.989999999999995</v>
       </c>
-      <c r="E68" s="19" t="s">
+      <c r="E68" s="13" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A69" s="11"/>
+      <c r="A69" s="22"/>
       <c r="B69" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C69" s="16" t="s">
+      <c r="C69" s="11" t="s">
         <v>199</v>
       </c>
       <c r="D69">
         <v>86.99</v>
       </c>
-      <c r="E69" s="19" t="s">
+      <c r="E69" s="13" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A70" s="11"/>
+      <c r="A70" s="22"/>
       <c r="B70" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C70" s="16" t="s">
+      <c r="C70" s="11" t="s">
         <v>201</v>
       </c>
       <c r="D70">
         <v>169</v>
       </c>
-      <c r="E70" s="19" t="s">
+      <c r="E70" s="13" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A71" s="11"/>
+      <c r="A71" s="22"/>
       <c r="B71" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C71" s="16" t="s">
+      <c r="C71" s="11" t="s">
         <v>203</v>
       </c>
       <c r="D71">
         <v>89.99</v>
       </c>
-      <c r="E71" s="19" t="s">
+      <c r="E71" s="13" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A72" s="11"/>
+      <c r="A72" s="22"/>
       <c r="B72" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C72" s="16" t="s">
+      <c r="C72" s="11" t="s">
         <v>205</v>
       </c>
       <c r="D72">
         <v>89.99</v>
       </c>
-      <c r="E72" s="19" t="s">
+      <c r="E72" s="13" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A73" s="11"/>
+      <c r="A73" s="22"/>
       <c r="B73" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C73" s="16" t="s">
+      <c r="C73" s="11" t="s">
         <v>207</v>
       </c>
       <c r="D73">
         <v>79.989999999999995</v>
       </c>
-      <c r="E73" s="19" t="s">
+      <c r="E73" s="13" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" s="14" t="s">
+      <c r="A74" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B74" s="15" t="s">
+      <c r="B74" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C74" s="12" t="s">
+      <c r="C74" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D74" s="12" t="s">
+      <c r="D74" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="E74" s="12" t="s">
+      <c r="E74" s="19" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="14"/>
-      <c r="B75" s="15"/>
-      <c r="C75" s="12"/>
-      <c r="D75" s="12"/>
-      <c r="E75" s="12"/>
+      <c r="A75" s="20"/>
+      <c r="B75" s="18"/>
+      <c r="C75" s="19"/>
+      <c r="D75" s="19"/>
+      <c r="E75" s="19"/>
     </row>
     <row r="76" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A76" s="11" t="s">
+      <c r="A76" s="22" t="s">
         <v>121</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C76" s="16" t="s">
+      <c r="C76" s="11" t="s">
         <v>209</v>
       </c>
       <c r="D76">
         <v>39.99</v>
       </c>
-      <c r="E76" s="19" t="s">
+      <c r="E76" s="13" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A77" s="11"/>
+      <c r="A77" s="22"/>
       <c r="B77" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C77" s="16" t="s">
+      <c r="C77" s="11" t="s">
         <v>211</v>
       </c>
       <c r="D77">
         <v>68.989999999999995</v>
       </c>
-      <c r="E77" s="19" t="s">
+      <c r="E77" s="13" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A78" s="11"/>
+      <c r="A78" s="22"/>
       <c r="B78" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C78" s="16" t="s">
+      <c r="C78" s="11" t="s">
         <v>213</v>
       </c>
       <c r="D78">
         <v>65.540000000000006</v>
       </c>
-      <c r="E78" s="19" t="s">
+      <c r="E78" s="13" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A79" s="11"/>
+      <c r="A79" s="22"/>
       <c r="B79" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C79" s="16" t="s">
+      <c r="C79" s="11" t="s">
         <v>215</v>
       </c>
       <c r="D79">
         <v>29.99</v>
       </c>
-      <c r="E79" s="19" t="s">
+      <c r="E79" s="13" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A80" s="11"/>
+      <c r="A80" s="22"/>
       <c r="B80" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C80" s="16" t="s">
+      <c r="C80" s="11" t="s">
         <v>217</v>
       </c>
       <c r="D80">
         <v>69.989999999999995</v>
       </c>
-      <c r="E80" s="19" t="s">
+      <c r="E80" s="13" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A81" s="11"/>
+      <c r="A81" s="22"/>
       <c r="B81" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C81" s="16" t="s">
+      <c r="C81" s="11" t="s">
         <v>219</v>
       </c>
       <c r="D81">
         <v>53.99</v>
       </c>
-      <c r="E81" s="19" t="s">
+      <c r="E81" s="13" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A82" s="11"/>
+      <c r="A82" s="22"/>
       <c r="B82" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C82" s="16" t="s">
+      <c r="C82" s="11" t="s">
         <v>221</v>
       </c>
       <c r="D82">
         <v>71.989999999999995</v>
       </c>
-      <c r="E82" s="19" t="s">
+      <c r="E82" s="13" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="14" t="s">
+      <c r="A83" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B83" s="15" t="s">
+      <c r="B83" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C83" s="12" t="s">
+      <c r="C83" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D83" s="12" t="s">
+      <c r="D83" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="E83" s="12" t="s">
+      <c r="E83" s="19" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="14"/>
-      <c r="B84" s="15"/>
-      <c r="C84" s="12"/>
-      <c r="D84" s="12"/>
-      <c r="E84" s="12"/>
+      <c r="A84" s="20"/>
+      <c r="B84" s="18"/>
+      <c r="C84" s="19"/>
+      <c r="D84" s="19"/>
+      <c r="E84" s="19"/>
     </row>
     <row r="85" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A85" s="11" t="s">
+      <c r="A85" s="22" t="s">
         <v>122</v>
       </c>
       <c r="B85" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C85" s="16" t="s">
+      <c r="C85" s="11" t="s">
         <v>223</v>
       </c>
       <c r="D85">
         <v>37.71</v>
       </c>
-      <c r="E85" s="19" t="s">
+      <c r="E85" s="13" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="86" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A86" s="11"/>
+      <c r="A86" s="22"/>
       <c r="B86" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C86" s="16" t="s">
+      <c r="C86" s="11" t="s">
         <v>225</v>
       </c>
       <c r="D86">
         <v>129.94999999999999</v>
       </c>
-      <c r="E86" s="19" t="s">
+      <c r="E86" s="13" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="87" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A87" s="11"/>
+      <c r="A87" s="22"/>
       <c r="B87" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C87" s="16" t="s">
+      <c r="C87" s="11" t="s">
         <v>227</v>
       </c>
       <c r="D87">
         <v>37.99</v>
       </c>
-      <c r="E87" s="19" t="s">
+      <c r="E87" s="13" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A88" s="11"/>
+      <c r="A88" s="22"/>
       <c r="B88" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C88" s="16" t="s">
+      <c r="C88" s="11" t="s">
         <v>229</v>
       </c>
       <c r="D88">
         <v>159.99</v>
       </c>
-      <c r="E88" s="19" t="s">
+      <c r="E88" s="13" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A89" s="11"/>
+      <c r="A89" s="22"/>
       <c r="B89" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C89" s="16" t="s">
+      <c r="C89" s="11" t="s">
         <v>231</v>
       </c>
       <c r="D89">
         <v>79.95</v>
       </c>
-      <c r="E89" s="19" t="s">
+      <c r="E89" s="13" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="90" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A90" s="11"/>
+      <c r="A90" s="22"/>
       <c r="B90" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C90" s="16" t="s">
+      <c r="C90" s="11" t="s">
         <v>233</v>
       </c>
       <c r="D90">
         <v>42.99</v>
       </c>
-      <c r="E90" s="19" t="s">
+      <c r="E90" s="13" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A91" s="11"/>
+      <c r="A91" s="22"/>
       <c r="B91" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C91" s="16" t="s">
+      <c r="C91" s="11" t="s">
         <v>235</v>
       </c>
       <c r="D91">
         <v>48.99</v>
       </c>
-      <c r="E91" s="19" t="s">
+      <c r="E91" s="13" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" s="14" t="s">
+      <c r="A92" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B92" s="15" t="s">
+      <c r="B92" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C92" s="12" t="s">
+      <c r="C92" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D92" s="12" t="s">
+      <c r="D92" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="E92" s="12" t="s">
+      <c r="E92" s="19" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" s="14"/>
-      <c r="B93" s="15"/>
-      <c r="C93" s="12"/>
-      <c r="D93" s="12"/>
-      <c r="E93" s="12"/>
+      <c r="A93" s="20"/>
+      <c r="B93" s="18"/>
+      <c r="C93" s="19"/>
+      <c r="D93" s="19"/>
+      <c r="E93" s="19"/>
     </row>
     <row r="94" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A94" s="11" t="s">
+      <c r="A94" s="22" t="s">
         <v>123</v>
       </c>
       <c r="B94" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C94" s="16" t="s">
+      <c r="C94" s="11" t="s">
         <v>237</v>
       </c>
       <c r="D94">
         <v>49.99</v>
       </c>
-      <c r="E94" s="19" t="s">
+      <c r="E94" s="13" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="95" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A95" s="11"/>
+      <c r="A95" s="22"/>
       <c r="B95" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C95" s="16" t="s">
+      <c r="C95" s="11" t="s">
         <v>239</v>
       </c>
       <c r="D95">
         <v>57.99</v>
       </c>
-      <c r="E95" s="19" t="s">
+      <c r="E95" s="13" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="96" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A96" s="11"/>
+      <c r="A96" s="22"/>
       <c r="B96" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C96" s="16" t="s">
+      <c r="C96" s="11" t="s">
         <v>241</v>
       </c>
       <c r="D96">
         <v>128.99</v>
       </c>
-      <c r="E96" s="19" t="s">
+      <c r="E96" s="13" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="97" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A97" s="11"/>
+      <c r="A97" s="22"/>
       <c r="B97" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C97" s="16" t="s">
+      <c r="C97" s="11" t="s">
         <v>243</v>
       </c>
       <c r="D97">
         <v>89.99</v>
       </c>
-      <c r="E97" s="19" t="s">
+      <c r="E97" s="13" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="98" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A98" s="11"/>
+      <c r="A98" s="22"/>
       <c r="B98" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C98" s="16" t="s">
+      <c r="C98" s="11" t="s">
         <v>245</v>
       </c>
       <c r="D98">
         <v>39.979999999999997</v>
       </c>
-      <c r="E98" s="19" t="s">
+      <c r="E98" s="13" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="99" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A99" s="11"/>
+      <c r="A99" s="22"/>
       <c r="B99" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C99" s="16" t="s">
+      <c r="C99" s="11" t="s">
         <v>247</v>
       </c>
       <c r="D99">
         <v>99.99</v>
       </c>
-      <c r="E99" s="19" t="s">
+      <c r="E99" s="13" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="100" spans="1:5" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A100" s="11"/>
+      <c r="A100" s="22"/>
       <c r="B100" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C100" s="16" t="s">
+      <c r="C100" s="11" t="s">
         <v>249</v>
       </c>
       <c r="D100">
         <v>35.99</v>
       </c>
-      <c r="E100" s="19" t="s">
+      <c r="E100" s="13" t="s">
         <v>250</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="86">
-    <mergeCell ref="B92:B93"/>
-    <mergeCell ref="C92:C93"/>
-    <mergeCell ref="D92:D93"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="E56:E57"/>
-    <mergeCell ref="E65:E66"/>
-    <mergeCell ref="E74:E75"/>
-    <mergeCell ref="E83:E84"/>
-    <mergeCell ref="E92:E93"/>
-    <mergeCell ref="B74:B75"/>
-    <mergeCell ref="C74:C75"/>
-    <mergeCell ref="D74:D75"/>
-    <mergeCell ref="A83:A84"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="C83:C84"/>
-    <mergeCell ref="D83:D84"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="A65:A66"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="C65:C66"/>
-    <mergeCell ref="D65:D66"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="B47:B48"/>
-    <mergeCell ref="C47:C48"/>
-    <mergeCell ref="D47:D48"/>
-    <mergeCell ref="L20:L21"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="D29:D30"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="H20:H21"/>
-    <mergeCell ref="I20:I21"/>
-    <mergeCell ref="J20:J21"/>
-    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="A85:A91"/>
+    <mergeCell ref="A94:A100"/>
+    <mergeCell ref="A31:A37"/>
+    <mergeCell ref="A40:A46"/>
+    <mergeCell ref="A49:A55"/>
+    <mergeCell ref="A58:A64"/>
+    <mergeCell ref="A67:A73"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="A56:A57"/>
+    <mergeCell ref="A74:A75"/>
+    <mergeCell ref="A92:A93"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="A22:A28"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="F20:F21"/>
     <mergeCell ref="K2:K3"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="F2:F3"/>
@@ -3101,34 +3088,49 @@
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="B11:B12"/>
     <mergeCell ref="C11:C12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="A22:A28"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C47:C48"/>
+    <mergeCell ref="D47:D48"/>
+    <mergeCell ref="L20:L21"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="D29:D30"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="H20:H21"/>
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="J20:J21"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="A83:A84"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="C83:C84"/>
+    <mergeCell ref="D83:D84"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="B65:B66"/>
+    <mergeCell ref="C65:C66"/>
+    <mergeCell ref="D65:D66"/>
     <mergeCell ref="A76:A82"/>
-    <mergeCell ref="A85:A91"/>
-    <mergeCell ref="A94:A100"/>
-    <mergeCell ref="A31:A37"/>
-    <mergeCell ref="A40:A46"/>
-    <mergeCell ref="A49:A55"/>
-    <mergeCell ref="A58:A64"/>
-    <mergeCell ref="A67:A73"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="A56:A57"/>
-    <mergeCell ref="A74:A75"/>
-    <mergeCell ref="A92:A93"/>
+    <mergeCell ref="B92:B93"/>
+    <mergeCell ref="C92:C93"/>
+    <mergeCell ref="D92:D93"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="E56:E57"/>
+    <mergeCell ref="E65:E66"/>
+    <mergeCell ref="E74:E75"/>
+    <mergeCell ref="E83:E84"/>
+    <mergeCell ref="E92:E93"/>
+    <mergeCell ref="B74:B75"/>
+    <mergeCell ref="C74:C75"/>
+    <mergeCell ref="D74:D75"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>

</xml_diff>